<commit_message>
Added unit testing for the ChequingAccount class.
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lauri\Desktop\Intermediate Software Development0315\2. Assignments\assignments\assignment_02\instructions\given_files\assignment_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Documents\rrc_polytech\winter_2025\isd_2025\Assignments\isd_project\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6021882D-84F4-49DA-9891-8E6AE904D6DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="3555" windowWidth="25185" windowHeight="11415" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="2400" yWindow="2655" windowWidth="21600" windowHeight="11295" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -249,6 +249,94 @@
   </si>
   <si>
     <t>Attributes are set to input values (ensure to test for superclass and subclass attributes)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account_number = 1234
+client_number = 1
+balance = 1000.0
+date_created = 1/1/2025
+overdraft_limit = -100
+overdraft_rate = 0.05
+</t>
+  </si>
+  <si>
+    <t>account_number = 1234
+client_number = 1
+balance = 1000.0
+date_created = 1/1/2025
+overdraft_limit = -100
+overdraft_rate = 0.05</t>
+  </si>
+  <si>
+    <t>balance = 1000.0</t>
+  </si>
+  <si>
+    <t>f"Account Number: 1234 Balance: $1,000.00\n
+Overdraft Limit: $-100.00 Overdraft Rate: 5.00% Account Type: Chequing"</t>
+  </si>
+  <si>
+    <t>Object initialized with the correct state</t>
+  </si>
+  <si>
+    <t>Object initialized with the correct state (overdraft_limit = -100)</t>
+  </si>
+  <si>
+    <t>Object initialized with the correct state (overdraft_rate = 0.05)</t>
+  </si>
+  <si>
+    <t>Object initialized with the correct state (date_created = date.today())</t>
+  </si>
+  <si>
+    <t>Xavier Balzer</t>
+  </si>
+  <si>
+    <t>"0.50"</t>
+  </si>
+  <si>
+    <t>"3"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account_number = 1234
+client_number = 1
+balance = 1000.0
+date_created = 1/1/2025
+overdraft_limit = -100
+overdraft_rate = "string"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account_number = 1234
+client_number = 1
+balance = 1000.0
+date_created = 1/1/2025
+overdraft_limit = "string"
+overdraft_rate = 0.05
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account_number = 1234
+client_number = 1
+balance = 1000.0
+date_created = "string"
+overdraft_limit = -100
+overdraft_rate = 0.05
+</t>
+  </si>
+  <si>
+    <t>account_number = 1234
+client_number = 1
+date_created = 1/1/2025
+overdraft_limit = -100
+overdraft_rate = 0.05</t>
+  </si>
+  <si>
+    <t>balance = -150</t>
+  </si>
+  <si>
+    <t>balance = -100</t>
   </si>
 </sst>
 </file>
@@ -555,7 +643,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -610,12 +698,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
     <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -629,12 +721,8 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1180,7 +1268,9 @@
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
+      <c r="C3" s="16" t="s">
+        <v>31</v>
+      </c>
       <c r="D3" s="17"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1225,9 +1315,15 @@
       <c r="D7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
+      <c r="E7" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
@@ -1239,9 +1335,15 @@
       <c r="D8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
+      <c r="E8" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="11">
@@ -1253,9 +1355,15 @@
       <c r="D9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="12"/>
+      <c r="E9" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="11">
@@ -1267,9 +1375,15 @@
       <c r="D10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="E10" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
@@ -1281,9 +1395,15 @@
       <c r="D11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
+      <c r="E11" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="12" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11">
@@ -1295,9 +1415,15 @@
       <c r="D12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+      <c r="E12" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="13" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="11">
@@ -1309,9 +1435,15 @@
       <c r="D13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
+      <c r="E13" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="14" spans="2:7" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
@@ -1323,9 +1455,15 @@
       <c r="D14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
+      <c r="E14" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="15" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="11">

</xml_diff>

<commit_message>
Created SavingsAccount class and __init__ method.
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Documents\rrc_polytech\winter_2025\isd_2025\Assignments\isd_project\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6021882D-84F4-49DA-9891-8E6AE904D6DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1FB17A-6D3B-4779-B442-4A6FACBB0F30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="2655" windowWidth="21600" windowHeight="11295" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -674,6 +674,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -697,9 +700,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1256,31 +1256,31 @@
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="17"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="19"/>
+      <c r="D4" s="20"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
@@ -1401,7 +1401,7 @@
       <c r="F11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="22" t="s">
+      <c r="G11" s="14" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1626,14 +1626,14 @@
       <c r="G30" s="5"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>